<commit_message>
feat: implement pharmacy purchase GRN popup modal with Excel template import/export, selling taxes mapping, and low stock threshold variables
</commit_message>
<xml_diff>
--- a/frontend/public/sample_inventory.xlsx
+++ b/frontend/public/sample_inventory.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Inventory Template" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,56 +397,59 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:Q5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Sno.</v>
+        <v>S.No</v>
       </c>
       <c r="B1" t="str">
-        <v>Item Name</v>
+        <v>Medicine Name</v>
       </c>
       <c r="C1" t="str">
-        <v>Old MRP</v>
+        <v>Description</v>
       </c>
       <c r="D1" t="str">
-        <v>Pack</v>
+        <v>Dosage Form</v>
       </c>
       <c r="E1" t="str">
-        <v>MRP</v>
+        <v>Pack Type</v>
       </c>
       <c r="F1" t="str">
-        <v>Quantity</v>
+        <v>Units / Pack</v>
       </c>
       <c r="G1" t="str">
-        <v>Free</v>
+        <v>Quantity (Packs)</v>
       </c>
       <c r="H1" t="str">
-        <v>Rate</v>
+        <v>Batch No</v>
       </c>
       <c r="I1" t="str">
-        <v>Dis</v>
+        <v>Expiry Date</v>
       </c>
       <c r="J1" t="str">
-        <v>Batch</v>
+        <v>Rate (Ex GST)</v>
       </c>
       <c r="K1" t="str">
-        <v>Expiry</v>
+        <v>Per Unit Rate</v>
       </c>
       <c r="L1" t="str">
-        <v>NRate</v>
+        <v>SGST %</v>
       </c>
       <c r="M1" t="str">
-        <v>HSN</v>
+        <v>CGST %</v>
       </c>
       <c r="N1" t="str">
-        <v>SGST</v>
+        <v>MRP (Inc GST)</v>
       </c>
       <c r="O1" t="str">
-        <v>CST</v>
+        <v>Per Unit Rate With GST</v>
       </c>
       <c r="P1" t="str">
-        <v>Amount</v>
+        <v>HSN Code</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Threshold Medicine Number</v>
       </c>
     </row>
     <row r="2">
@@ -456,47 +459,50 @@
       <c r="B2" t="str">
         <v>Paracetamol 500mg</v>
       </c>
-      <c r="C2">
-        <v>15</v>
+      <c r="C2" t="str">
+        <v>Analgesic and antipyretic</v>
       </c>
       <c r="D2" t="str">
-        <v>10 Tab</v>
-      </c>
-      <c r="E2">
-        <v>20</v>
+        <v>Tablet</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Strip</v>
       </c>
       <c r="F2">
-        <v>200</v>
+        <v>10</v>
       </c>
       <c r="G2">
         <v>20</v>
       </c>
-      <c r="H2">
-        <v>10</v>
-      </c>
-      <c r="I2">
-        <v>5</v>
-      </c>
-      <c r="J2" t="str">
+      <c r="H2" t="str">
         <v>B123</v>
       </c>
-      <c r="K2" t="str">
-        <v>05/2028</v>
+      <c r="I2" t="str">
+        <v>2028-12-31</v>
+      </c>
+      <c r="J2">
+        <v>80</v>
+      </c>
+      <c r="K2">
+        <v>8</v>
       </c>
       <c r="L2">
-        <v>9.5</v>
-      </c>
-      <c r="M2" t="str">
-        <v>3004</v>
+        <v>6</v>
+      </c>
+      <c r="M2">
+        <v>6</v>
       </c>
       <c r="N2">
-        <v>6</v>
+        <v>96</v>
       </c>
       <c r="O2">
-        <v>6</v>
-      </c>
-      <c r="P2">
-        <v>2000</v>
+        <v>9.6</v>
+      </c>
+      <c r="P2" t="str">
+        <v>30049011</v>
+      </c>
+      <c r="Q2">
+        <v>50</v>
       </c>
     </row>
     <row r="3">
@@ -506,47 +512,50 @@
       <c r="B3" t="str">
         <v>Amoxicillin 250mg</v>
       </c>
-      <c r="C3">
-        <v>45</v>
+      <c r="C3" t="str">
+        <v>Antibiotic medication</v>
       </c>
       <c r="D3" t="str">
-        <v>10 Tab</v>
-      </c>
-      <c r="E3">
-        <v>50</v>
+        <v>Capsule</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Strip</v>
       </c>
       <c r="F3">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="G3">
-        <v>0</v>
-      </c>
-      <c r="H3">
-        <v>35</v>
-      </c>
-      <c r="I3">
-        <v>10</v>
-      </c>
-      <c r="J3" t="str">
+        <v>3</v>
+      </c>
+      <c r="H3" t="str">
         <v>AM99</v>
       </c>
-      <c r="K3" t="str">
-        <v>08/2027</v>
+      <c r="I3" t="str">
+        <v>2027-08-15</v>
+      </c>
+      <c r="J3">
+        <v>120</v>
+      </c>
+      <c r="K3">
+        <v>12</v>
       </c>
       <c r="L3">
-        <v>31.5</v>
-      </c>
-      <c r="M3" t="str">
-        <v>3004</v>
+        <v>6</v>
+      </c>
+      <c r="M3">
+        <v>6</v>
       </c>
       <c r="N3">
-        <v>6</v>
+        <v>144</v>
       </c>
       <c r="O3">
-        <v>6</v>
-      </c>
-      <c r="P3">
-        <v>1050</v>
+        <v>14.4</v>
+      </c>
+      <c r="P3" t="str">
+        <v>30041010</v>
+      </c>
+      <c r="Q3">
+        <v>40</v>
       </c>
     </row>
     <row r="4">
@@ -556,47 +565,50 @@
       <c r="B4" t="str">
         <v>Ibuprofen 400mg</v>
       </c>
-      <c r="C4">
-        <v>12</v>
+      <c r="C4" t="str">
+        <v>NSAID pain reliever</v>
       </c>
       <c r="D4" t="str">
-        <v>10 Tab</v>
-      </c>
-      <c r="E4">
+        <v>Tablet</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Strip</v>
+      </c>
+      <c r="F4">
+        <v>10</v>
+      </c>
+      <c r="G4">
         <v>15</v>
       </c>
-      <c r="F4">
-        <v>150</v>
-      </c>
-      <c r="G4">
-        <v>10</v>
-      </c>
-      <c r="H4">
-        <v>8</v>
-      </c>
-      <c r="I4">
-        <v>0</v>
-      </c>
-      <c r="J4" t="str">
+      <c r="H4" t="str">
         <v>IB11</v>
       </c>
-      <c r="K4" t="str">
-        <v>07/2026</v>
+      <c r="I4" t="str">
+        <v>2027-07-20</v>
+      </c>
+      <c r="J4">
+        <v>40</v>
+      </c>
+      <c r="K4">
+        <v>4</v>
       </c>
       <c r="L4">
-        <v>8</v>
-      </c>
-      <c r="M4" t="str">
-        <v>3004</v>
+        <v>6</v>
+      </c>
+      <c r="M4">
+        <v>6</v>
       </c>
       <c r="N4">
-        <v>6</v>
+        <v>48</v>
       </c>
       <c r="O4">
-        <v>6</v>
-      </c>
-      <c r="P4">
-        <v>1200</v>
+        <v>4.8</v>
+      </c>
+      <c r="P4" t="str">
+        <v>30049099</v>
+      </c>
+      <c r="Q4">
+        <v>100</v>
       </c>
     </row>
     <row r="5">
@@ -606,52 +618,55 @@
       <c r="B5" t="str">
         <v>Vitamin C Chews</v>
       </c>
-      <c r="C5">
+      <c r="C5" t="str">
+        <v>Vitamin supplement</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Chewable</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Bottle</v>
+      </c>
+      <c r="F5">
         <v>30</v>
-      </c>
-      <c r="D5" t="str">
-        <v>15 Tab</v>
-      </c>
-      <c r="E5">
-        <v>35</v>
-      </c>
-      <c r="F5">
-        <v>25</v>
       </c>
       <c r="G5">
         <v>5</v>
       </c>
-      <c r="H5">
-        <v>20</v>
-      </c>
-      <c r="I5">
-        <v>0</v>
-      </c>
-      <c r="J5" t="str">
+      <c r="H5" t="str">
         <v>VT01</v>
       </c>
-      <c r="K5" t="str">
-        <v>05/2026</v>
+      <c r="I5" t="str">
+        <v>2026-11-30</v>
+      </c>
+      <c r="J5">
+        <v>150</v>
+      </c>
+      <c r="K5">
+        <v>5</v>
       </c>
       <c r="L5">
-        <v>20</v>
-      </c>
-      <c r="M5" t="str">
-        <v>3004</v>
+        <v>6</v>
+      </c>
+      <c r="M5">
+        <v>6</v>
       </c>
       <c r="N5">
-        <v>6</v>
+        <v>180</v>
       </c>
       <c r="O5">
         <v>6</v>
       </c>
-      <c r="P5">
-        <v>500</v>
+      <c r="P5" t="str">
+        <v>29362700</v>
+      </c>
+      <c r="Q5">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>